<commit_message>
ci: configuration du pipeline de sécurité avec SynK 1
</commit_message>
<xml_diff>
--- a/Journal_Amelioration.xlsx
+++ b/Journal_Amelioration.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14388" uniqueCount="728">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24768" uniqueCount="740">
   <si>
     <t xml:space="preserve">Identification du document </t>
   </si>
@@ -2248,6 +2248,42 @@
   </si>
   <si>
     <t>rrrrrr</t>
+  </si>
+  <si>
+    <t>#215</t>
+  </si>
+  <si>
+    <t>eeee</t>
+  </si>
+  <si>
+    <t>29/04/2026</t>
+  </si>
+  <si>
+    <t>rrrr</t>
+  </si>
+  <si>
+    <t>Constat d'audit : dddd</t>
+  </si>
+  <si>
+    <t>#216</t>
+  </si>
+  <si>
+    <t>zzz</t>
+  </si>
+  <si>
+    <t>Constat d'audit : eeeee</t>
+  </si>
+  <si>
+    <t>#217</t>
+  </si>
+  <si>
+    <t>ccc</t>
+  </si>
+  <si>
+    <t>Constat d'audit : ccc</t>
+  </si>
+  <si>
+    <t>12/04/2026</t>
   </si>
 </sst>
 </file>
@@ -4601,7 +4637,7 @@
   <sheetPr filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N221"/>
+  <dimension ref="A1:N224"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" customWidth="true" style="9" width="10.42578125"/>
@@ -13851,7 +13887,7 @@
         <v>612</v>
       </c>
       <c r="K220" t="s" s="19">
-        <v>719</v>
+        <v>739</v>
       </c>
       <c r="L220" t="s" s="18">
         <v>719</v>
@@ -13892,6 +13928,120 @@
         <v>719</v>
       </c>
       <c r="L221" t="s" s="18">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="s" s="9">
+        <v>728</v>
+      </c>
+      <c r="B222" t="s" s="13">
+        <v>729</v>
+      </c>
+      <c r="C222" t="s" s="21">
+        <v>531</v>
+      </c>
+      <c r="D222" t="s" s="9">
+        <v>531</v>
+      </c>
+      <c r="E222" t="s" s="9">
+        <v>730</v>
+      </c>
+      <c r="F222" t="s" s="9">
+        <v>531</v>
+      </c>
+      <c r="G222" t="s" s="9">
+        <v>731</v>
+      </c>
+      <c r="H222" t="s" s="9">
+        <v>531</v>
+      </c>
+      <c r="I222" t="s" s="20">
+        <v>732</v>
+      </c>
+      <c r="J222" t="s" s="16">
+        <v>612</v>
+      </c>
+      <c r="K222" t="s" s="19">
+        <v>719</v>
+      </c>
+      <c r="L222" t="s" s="18">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="s" s="9">
+        <v>733</v>
+      </c>
+      <c r="B223" t="s" s="13">
+        <v>734</v>
+      </c>
+      <c r="C223" t="s" s="21">
+        <v>531</v>
+      </c>
+      <c r="D223" t="s" s="9">
+        <v>531</v>
+      </c>
+      <c r="E223" t="s" s="9">
+        <v>730</v>
+      </c>
+      <c r="F223" t="s" s="9">
+        <v>531</v>
+      </c>
+      <c r="G223" t="s" s="9">
+        <v>734</v>
+      </c>
+      <c r="H223" t="s" s="9">
+        <v>531</v>
+      </c>
+      <c r="I223" t="s" s="20">
+        <v>735</v>
+      </c>
+      <c r="J223" t="s" s="16">
+        <v>612</v>
+      </c>
+      <c r="K223" t="s" s="19">
+        <v>719</v>
+      </c>
+      <c r="L223" t="s" s="18">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="s" s="9">
+        <v>736</v>
+      </c>
+      <c r="B224" t="s" s="13">
+        <v>737</v>
+      </c>
+      <c r="C224" t="s" s="21">
+        <v>531</v>
+      </c>
+      <c r="D224" t="s" s="9">
+        <v>531</v>
+      </c>
+      <c r="E224" t="s" s="9">
+        <v>730</v>
+      </c>
+      <c r="F224" t="s" s="9">
+        <v>531</v>
+      </c>
+      <c r="G224" t="s" s="9">
+        <v>737</v>
+      </c>
+      <c r="H224" t="s" s="9">
+        <v>531</v>
+      </c>
+      <c r="I224" t="s" s="20">
+        <v>738</v>
+      </c>
+      <c r="J224" t="s" s="16">
+        <v>612</v>
+      </c>
+      <c r="K224" t="s" s="19">
+        <v>719</v>
+      </c>
+      <c r="L224" t="s" s="18">
         <v>719</v>
       </c>
     </row>

</xml_diff>